<commit_message>
Update RTS-GMLC to new investcost (from Frauental translators)
</commit_message>
<xml_diff>
--- a/data/RTS-GMLC/Data_Sources.xlsx
+++ b/data/RTS-GMLC/Data_Sources.xlsx
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.5703125" customWidth="1" min="1" max="1"/>
@@ -1072,17 +1072,17 @@
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>RTS-GMLC-storage-placeholder</t>
+          <t>RTS-GMLC-storage-battery-ise</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>gen.csv, storage.csv, bus.csv</t>
+          <t>gen.csv, storage.csv, bus.csv; InvestCost: Fraunhofer ISE 'Studie Stromgestehungskosten Erneuerbare Energien 2024'</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>BSD 3-Clause</t>
+          <t>BSD 3-Clause (RTS-GMLC data); Public (investment cost)</t>
         </is>
       </c>
       <c r="F17" s="11" t="inlineStr">
@@ -1092,12 +1092,12 @@
       </c>
       <c r="G17" s="11" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>DisEffic=ChEffic=sqrt(Roundtrip Efficiency / 100) - symmetric split; Ene2PowRatio=Max Volume [MWh] / MaxProd [MW]; IniReserve=Initial Volume / Max Volume; HYDRO and CSP: gen.csv stores 0 for roundtrip efficiency (field not populated in RTS-GMLC) - defaulted to 1.0. InvestCost (Battery, CSP thermal storage): Placeholder investment cost - can be updated in future with real-world cost. Per-generator ±0.5 % deterministic variation applied to prevent degenerate optimisation.</t>
+          <t>DisEffic=ChEffic=sqrt(Roundtrip Efficiency / 100) - symmetric split; Ene2PowRatio=Max Volume [MWh] / MaxProd [MW]; IniReserve=Initial Volume / Max Volume; HYDRO and CSP: gen.csv stores 0 for roundtrip efficiency (field not populated in RTS-GMLC) - defaulted to 1.0. InvestCost (Battery 313_STORAGE_1): InvestCostPerMWh from Fraunhofer ISE 'Studie Stromgestehungskosten Erneuerbare Energien 2024', Tabelle 1 'Batteriespeicher für PV-Freiflächenanlagen' (400-600 EUR/kWh usable capacity incl. installation, average 500) divided by the 15-year battery lifetime of Tabelle 2 (battery replacement cost not included); InvestCostPerMW fixed at 0 (ISE gives no separate power cost). The ±0.5 % variation is applied to InvestCostPerMWh.</t>
         </is>
       </c>
     </row>
@@ -1107,12 +1107,12 @@
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>RTS-GMLC-load</t>
+          <t>RTS-GMLC-storage-placeholder</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>bus.csv, REAL_TIME_regional_Load.csv, DAY_AHEAD_regional_Load.csv</t>
+          <t>gen.csv, storage.csv, bus.csv</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -1127,12 +1127,12 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>Area-level load disaggregated to buses using static MW Load shares from bus.csv; RT 5-min data aggregated to hourly arithmetic mean; DA 1-h forecast used as-is</t>
+          <t>DisEffic=ChEffic=sqrt(Roundtrip Efficiency / 100) - symmetric split; Ene2PowRatio=Max Volume [MWh] / MaxProd [MW]; IniReserve=Initial Volume / Max Volume; HYDRO and CSP: gen.csv stores 0 for roundtrip efficiency (field not populated in RTS-GMLC) - defaulted to 1.0. InvestCost (CSP thermal storage): Placeholder investment cost - can be updated in future with real-world cost. Per-generator ±0.5 % deterministic variation applied to prevent degenerate optimisation.</t>
         </is>
       </c>
     </row>
@@ -1142,12 +1142,12 @@
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>RTS-GMLC-ts-vres</t>
+          <t>RTS-GMLC-load</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>REAL_TIME/DAY_AHEAD pv.csv, rtpv.csv, wind.csv, Natural_Inflow.csv, hydro.csv</t>
+          <t>bus.csv, REAL_TIME_regional_Load.csv, DAY_AHEAD_regional_Load.csv</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="H19" s="11" t="inlineStr">
         <is>
-          <t>Timeseries [MW] divided by PMax and clipped to [0, 1]; RT 5-min data aggregated to hourly arithmetic mean; CSP solar-field output from Natural Inflow timeseries; ROR (201_HYDRO_4) from hydro timeseries</t>
+          <t>Area-level load disaggregated to buses using static MW Load shares from bus.csv; RT 5-min data aggregated to hourly arithmetic mean; DA 1-h forecast used as-is</t>
         </is>
       </c>
     </row>
@@ -1177,12 +1177,12 @@
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>RTS-GMLC-ts-inflows</t>
+          <t>RTS-GMLC-ts-vres</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>REAL_TIME/DAY_AHEAD hydro_inflow.csv</t>
+          <t>REAL_TIME/DAY_AHEAD pv.csv, rtpv.csv, wind.csv, Natural_Inflow.csv, hydro.csv</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>Column suffix _RESERVOIR_head stripped to recover GEN UID; RT 5-min data aggregated to hourly arithmetic mean; ROR unit (201_HYDRO_4) excluded (handled via Power_VRESProfiles)</t>
+          <t>Timeseries [MW] divided by PMax and clipped to [0, 1]; RT 5-min data aggregated to hourly arithmetic mean; CSP solar-field output from Natural Inflow timeseries; ROR (201_HYDRO_4) from hydro timeseries</t>
         </is>
       </c>
     </row>
@@ -1212,26 +1212,61 @@
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
+          <t>RTS-GMLC-ts-inflows</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>REAL_TIME/DAY_AHEAD hydro_inflow.csv</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>BSD 3-Clause</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>Felix Auer</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="H21" s="11" t="inlineStr">
+        <is>
+          <t>Column suffix _RESERVOIR_head stripped to recover GEN UID; RT 5-min data aggregated to hourly arithmetic mean; ROR unit (201_HYDRO_4) excluded (handled via Power_VRESProfiles)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="10" t="n">
+        <v/>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
           <t>RTS-GMLC-structure</t>
         </is>
       </c>
-      <c r="D21" s="11" t="n">
-        <v/>
-      </c>
-      <c r="E21" s="11" t="n">
-        <v/>
-      </c>
-      <c r="F21" s="11" t="inlineStr">
-        <is>
-          <t>Felix Auer</t>
-        </is>
-      </c>
-      <c r="G21" s="11" t="inlineStr">
+      <c r="D22" s="11" t="n">
+        <v/>
+      </c>
+      <c r="E22" s="11" t="n">
+        <v/>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>Felix Auer</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
         <is>
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="H21" s="11" t="inlineStr">
+      <c r="H22" s="11" t="inlineStr">
         <is>
           <t>Temporal structure not sourced from RTS-GMLC SourceData: 8784-hour representative period for 2020 (leap year), all timestep weights = 1.0 h, identity mapping p -&gt; (rp01, k)</t>
         </is>

</xml_diff>